<commit_message>
got printing to 7 segment display working
</commit_message>
<xml_diff>
--- a/Firmware/Other/segment layout.xlsx
+++ b/Firmware/Other/segment layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indesignllc1-my.sharepoint.com/personal/adwolfe_indesign-llc_com/Documents/M_Drive/Github/Home-Audio-System/Firmware/Other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{5C606BC9-FF45-4673-A1AC-2DE2D026D232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D4DEAD4-A070-4F4F-95C3-B7824A1AB438}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{5C606BC9-FF45-4673-A1AC-2DE2D026D232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C38AF600-912A-47E4-AA1D-BBA2D87FAE22}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
   <si>
     <t>OUT0</t>
   </si>
@@ -330,6 +330,12 @@
   </si>
   <si>
     <t>0x00</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>0x75</t>
   </si>
 </sst>
 </file>
@@ -1136,8 +1142,11 @@
       <c r="M16" t="s">
         <v>96</v>
       </c>
+      <c r="N16" t="s">
+        <v>98</v>
+      </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>88</v>
       </c>
@@ -1174,13 +1183,16 @@
       <c r="M17" t="s">
         <v>97</v>
       </c>
+      <c r="N17" t="s">
+        <v>99</v>
+      </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>75</v>
       </c>

</xml_diff>

<commit_message>
handle refresh in loop, set by flag in interrupt. Display eq value differently, and set based on dB table
</commit_message>
<xml_diff>
--- a/Firmware/Other/segment layout.xlsx
+++ b/Firmware/Other/segment layout.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indesignllc1-my.sharepoint.com/personal/adwolfe_indesign-llc_com/Documents/M_Drive/Github/Home-Audio-System/Firmware/Other/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69f5ad8fb782b24f/Documents/GitHub/Home-Audio-System/Firmware/Other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{5C606BC9-FF45-4673-A1AC-2DE2D026D232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C38AF600-912A-47E4-AA1D-BBA2D87FAE22}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{5C606BC9-FF45-4673-A1AC-2DE2D026D232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A759C13B-94C0-4EF3-950E-B0024B699726}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19905" yWindow="1155" windowWidth="15420" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="83">
   <si>
     <t>OUT0</t>
   </si>
@@ -143,15 +143,6 @@
     <t>0x76</t>
   </si>
   <si>
-    <t>0x44</t>
-  </si>
-  <si>
-    <t>0x7A</t>
-  </si>
-  <si>
-    <t>0x4C</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
@@ -182,60 +173,18 @@
     <t>o</t>
   </si>
   <si>
-    <t>0xDE</t>
-  </si>
-  <si>
     <t>0x6E</t>
   </si>
   <si>
     <t>0x64</t>
   </si>
   <si>
-    <t>0xEC</t>
-  </si>
-  <si>
-    <t>0x56</t>
-  </si>
-  <si>
-    <t>0x88</t>
-  </si>
-  <si>
-    <t>0xF4</t>
-  </si>
-  <si>
-    <t>0xF8</t>
-  </si>
-  <si>
-    <t>0xCA</t>
-  </si>
-  <si>
     <t>0x7E</t>
   </si>
   <si>
-    <t>0x98</t>
-  </si>
-  <si>
-    <t>0xFE</t>
-  </si>
-  <si>
-    <t>0xFA</t>
-  </si>
-  <si>
-    <t>0xBE</t>
-  </si>
-  <si>
-    <t>0xCE</t>
-  </si>
-  <si>
     <t>0x24</t>
   </si>
   <si>
-    <t>0xA8</t>
-  </si>
-  <si>
-    <t>0x6C</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
@@ -251,15 +200,9 @@
     <t>u</t>
   </si>
   <si>
-    <t>0xD6</t>
-  </si>
-  <si>
     <t>0x66</t>
   </si>
   <si>
-    <t>0x2C</t>
-  </si>
-  <si>
     <t>add one to any character value to engage the decimal point</t>
   </si>
   <si>
@@ -336,6 +279,12 @@
   </si>
   <si>
     <t>0x75</t>
+  </si>
+  <si>
+    <t>neg sign</t>
+  </si>
+  <si>
+    <t>0x02</t>
   </si>
 </sst>
 </file>
@@ -708,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:R20"/>
+  <dimension ref="A2:R15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
@@ -818,386 +767,211 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
         <v>21</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G8" t="s">
         <v>22</v>
       </c>
-      <c r="I6">
+      <c r="I8">
         <v>1</v>
       </c>
-      <c r="J6">
+      <c r="J8">
         <v>2</v>
       </c>
-      <c r="K6">
+      <c r="K8">
         <v>3</v>
       </c>
-      <c r="L6">
+      <c r="L8">
         <v>4</v>
       </c>
-      <c r="M6">
+      <c r="M8">
         <v>5</v>
       </c>
-      <c r="N6">
+      <c r="N8">
         <v>6</v>
       </c>
-      <c r="O6">
+      <c r="O8">
         <v>7</v>
       </c>
-      <c r="P6">
+      <c r="P8">
         <v>8</v>
       </c>
-      <c r="Q6">
+      <c r="Q8">
         <v>9</v>
       </c>
-      <c r="R6">
+      <c r="R8">
         <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" t="s">
-        <v>55</v>
-      </c>
-      <c r="L7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M7" t="s">
-        <v>36</v>
-      </c>
-      <c r="N7" t="s">
-        <v>57</v>
-      </c>
-      <c r="O7" t="s">
-        <v>58</v>
-      </c>
-      <c r="P7" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>60</v>
-      </c>
-      <c r="R7" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
         <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
         <v>45</v>
       </c>
       <c r="G9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" t="s">
+        <v>62</v>
+      </c>
+      <c r="L9" t="s">
+        <v>63</v>
+      </c>
+      <c r="M9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N9" t="s">
         <v>47</v>
       </c>
-      <c r="H9" t="s">
+      <c r="O9" t="s">
+        <v>65</v>
+      </c>
+      <c r="P9" t="s">
         <v>66</v>
       </c>
-      <c r="I9" t="s">
+      <c r="Q9" t="s">
         <v>67</v>
       </c>
-      <c r="J9" t="s">
+      <c r="R9" t="s">
         <v>68</v>
       </c>
-      <c r="K9" t="s">
-        <v>69</v>
-      </c>
-      <c r="L9" t="s">
-        <v>70</v>
-      </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10" t="s">
-        <v>71</v>
-      </c>
-      <c r="I10" t="s">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>35</v>
       </c>
-      <c r="J10" t="s">
+      <c r="C11" t="s">
         <v>36</v>
       </c>
-      <c r="K10" t="s">
-        <v>72</v>
-      </c>
-      <c r="L10" t="s">
-        <v>73</v>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" t="s">
+        <v>79</v>
+      </c>
+      <c r="P11" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I12" t="s">
+        <v>74</v>
+      </c>
+      <c r="J12" t="s">
+        <v>64</v>
+      </c>
+      <c r="K12" t="s">
+        <v>54</v>
+      </c>
+      <c r="L12" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E13" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13">
-        <v>1</v>
-      </c>
-      <c r="J13">
-        <v>2</v>
-      </c>
-      <c r="K13">
-        <v>3</v>
-      </c>
-      <c r="L13">
-        <v>4</v>
-      </c>
-      <c r="M13">
-        <v>5</v>
-      </c>
-      <c r="N13">
-        <v>6</v>
-      </c>
-      <c r="O13">
-        <v>7</v>
-      </c>
-      <c r="P13">
-        <v>8</v>
-      </c>
-      <c r="Q13">
-        <v>9</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
+      <c r="M12" t="s">
+        <v>78</v>
+      </c>
+      <c r="N12" t="s">
+        <v>80</v>
+      </c>
+      <c r="P12" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>33</v>
-      </c>
       <c r="B14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
         <v>76</v>
-      </c>
-      <c r="C14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" t="s">
-        <v>49</v>
-      </c>
-      <c r="G14" t="s">
-        <v>78</v>
-      </c>
-      <c r="I14" t="s">
-        <v>79</v>
-      </c>
-      <c r="J14" t="s">
-        <v>80</v>
-      </c>
-      <c r="K14" t="s">
-        <v>81</v>
-      </c>
-      <c r="L14" t="s">
-        <v>82</v>
-      </c>
-      <c r="M14" t="s">
-        <v>83</v>
-      </c>
-      <c r="N14" t="s">
-        <v>57</v>
-      </c>
-      <c r="O14" t="s">
-        <v>84</v>
-      </c>
-      <c r="P14" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>86</v>
-      </c>
-      <c r="R14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" t="s">
-        <v>44</v>
-      </c>
-      <c r="F16" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" t="s">
-        <v>47</v>
-      </c>
-      <c r="H16" t="s">
-        <v>66</v>
-      </c>
-      <c r="I16" t="s">
-        <v>67</v>
-      </c>
-      <c r="J16" t="s">
-        <v>68</v>
-      </c>
-      <c r="K16" t="s">
-        <v>69</v>
-      </c>
-      <c r="L16" t="s">
-        <v>70</v>
-      </c>
-      <c r="M16" t="s">
-        <v>96</v>
-      </c>
-      <c r="N16" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" t="s">
-        <v>50</v>
-      </c>
-      <c r="F17" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" t="s">
-        <v>91</v>
-      </c>
-      <c r="H17" t="s">
-        <v>92</v>
-      </c>
-      <c r="I17" t="s">
-        <v>93</v>
-      </c>
-      <c r="J17" t="s">
-        <v>83</v>
-      </c>
-      <c r="K17" t="s">
-        <v>72</v>
-      </c>
-      <c r="L17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M17" t="s">
-        <v>97</v>
-      </c>
-      <c r="N17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>75</v>
-      </c>
-      <c r="B20" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>